<commit_message>
Prepare MedSaathi for production deployment
</commit_message>
<xml_diff>
--- a/backend/data/medical_master.xlsx
+++ b/backend/data/medical_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/aaba9b7fc384692a/Desktop/Ai_medical_assitant/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{7313785C-7652-4BB8-BD78-FC04FC8A3E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05705764-9340-45AC-A0C4-59BF17ECD085}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{7313785C-7652-4BB8-BD78-FC04FC8A3E81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58FEEBCA-3AE0-4015-BBFE-B21B2E4047B6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0E185D9D-9B36-489F-B026-23D5259A59E6}"/>
   </bookViews>
@@ -10432,12 +10432,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -10452,8 +10458,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11629,7 +11636,7 @@
       <c r="C20" t="s">
         <v>107</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="1" t="s">
         <v>108</v>
       </c>
       <c r="E20" t="s">

</xml_diff>